<commit_message>
add: analysis code and figure
</commit_message>
<xml_diff>
--- a/saved/run_batch_20260912/analysis/v4_metrics_summary_plain.xlsx
+++ b/saved/run_batch_20260912/analysis/v4_metrics_summary_plain.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="v4_metrics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v4_metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
modify: reference candidate selection logic
</commit_message>
<xml_diff>
--- a/saved/run_batch_20260912/analysis/v4_metrics_summary_plain.xlsx
+++ b/saved/run_batch_20260912/analysis/v4_metrics_summary_plain.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,35 +454,50 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>jaccard_rigid</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>precision_rigid</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>recall_rigid</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>ias</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>turn_count</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>turn_to_1st_correct</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>turn_to_1st_confident</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>overcommitment_turns</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>overcommitment_conf</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>diagnostic_reasoning_overall_score</t>
         </is>
@@ -517,24 +532,33 @@
         <v>0.415893475877193</v>
       </c>
       <c r="H2" t="n">
+        <v>0.3792011513157895</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.5264231359649123</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.534404221491228</v>
+      </c>
+      <c r="K2" t="n">
         <v>0.4161504717057321</v>
       </c>
-      <c r="I2" t="n">
+      <c r="L2" t="n">
         <v>10.57391304347826</v>
       </c>
-      <c r="J2" t="n">
+      <c r="M2" t="n">
         <v>8.15072463768116</v>
       </c>
-      <c r="K2" t="n">
+      <c r="N2" t="n">
         <v>8.86376811594203</v>
       </c>
-      <c r="L2" t="n">
+      <c r="O2" t="n">
         <v>3.568115942028986</v>
       </c>
-      <c r="M2" t="n">
+      <c r="P2" t="n">
         <v>2.365217391304348</v>
       </c>
-      <c r="N2" t="n">
+      <c r="Q2" t="n">
         <v>0.7026315942028986</v>
       </c>
     </row>
@@ -567,24 +591,33 @@
         <v>0.392438845144357</v>
       </c>
       <c r="H3" t="n">
+        <v>0.407340780839895</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.5897354002624672</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.4917096456692913</v>
+      </c>
+      <c r="K3" t="n">
         <v>0.3859828345496255</v>
       </c>
-      <c r="I3" t="n">
+      <c r="L3" t="n">
         <v>8.834782608695653</v>
       </c>
-      <c r="J3" t="n">
+      <c r="M3" t="n">
         <v>7.15072463768116</v>
       </c>
-      <c r="K3" t="n">
+      <c r="N3" t="n">
         <v>7.304347826086956</v>
       </c>
-      <c r="L3" t="n">
+      <c r="O3" t="n">
         <v>2.768115942028985</v>
       </c>
-      <c r="M3" t="n">
+      <c r="P3" t="n">
         <v>2.150724637681159</v>
       </c>
-      <c r="N3" t="n">
+      <c r="Q3" t="n">
         <v>0.691099420289855</v>
       </c>
     </row>
@@ -617,24 +650,33 @@
         <v>0.3917180627047263</v>
       </c>
       <c r="H4" t="n">
+        <v>0.3967591951333646</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.5684520355638746</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.512912915301825</v>
+      </c>
+      <c r="K4" t="n">
         <v>0.463501933647481</v>
       </c>
-      <c r="I4" t="n">
+      <c r="L4" t="n">
         <v>6.194202898550724</v>
       </c>
-      <c r="J4" t="n">
+      <c r="M4" t="n">
         <v>5.704347826086956</v>
       </c>
-      <c r="K4" t="n">
+      <c r="N4" t="n">
         <v>5.87536231884058</v>
       </c>
-      <c r="L4" t="n">
+      <c r="O4" t="n">
         <v>1.385507246376812</v>
       </c>
-      <c r="M4" t="n">
+      <c r="P4" t="n">
         <v>0.9739130434782609</v>
       </c>
-      <c r="N4" t="n">
+      <c r="Q4" t="n">
         <v>0.6727484057971015</v>
       </c>
     </row>
@@ -667,24 +709,33 @@
         <v>0.3599038198632891</v>
       </c>
       <c r="H5" t="n">
+        <v>0.4305111781262566</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.6540267390430238</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.488223763570567</v>
+      </c>
+      <c r="K5" t="n">
         <v>0.4163217380664769</v>
       </c>
-      <c r="I5" t="n">
+      <c r="L5" t="n">
         <v>7.208695652173913</v>
       </c>
-      <c r="J5" t="n">
+      <c r="M5" t="n">
         <v>6.257971014492754</v>
       </c>
-      <c r="K5" t="n">
+      <c r="N5" t="n">
         <v>6.359420289855072</v>
       </c>
-      <c r="L5" t="n">
+      <c r="O5" t="n">
         <v>1.855072463768116</v>
       </c>
-      <c r="M5" t="n">
+      <c r="P5" t="n">
         <v>1.478260869565217</v>
       </c>
-      <c r="N5" t="n">
+      <c r="Q5" t="n">
         <v>0.6466733333333333</v>
       </c>
     </row>
@@ -717,24 +768,33 @@
         <v>0.4316124686192468</v>
       </c>
       <c r="H6" t="n">
+        <v>0.4298293723849372</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.6505427615062761</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.5154064435146444</v>
+      </c>
+      <c r="K6" t="n">
         <v>0.4584506540095213</v>
       </c>
-      <c r="I6" t="n">
+      <c r="L6" t="n">
         <v>6.927536231884058</v>
       </c>
-      <c r="J6" t="n">
+      <c r="M6" t="n">
         <v>5.855072463768116</v>
       </c>
-      <c r="K6" t="n">
+      <c r="N6" t="n">
         <v>5.991304347826087</v>
       </c>
-      <c r="L6" t="n">
+      <c r="O6" t="n">
         <v>1.776811594202899</v>
       </c>
-      <c r="M6" t="n">
+      <c r="P6" t="n">
         <v>1.542028985507246</v>
       </c>
-      <c r="N6" t="n">
+      <c r="Q6" t="n">
         <v>0.6801655072463768</v>
       </c>
     </row>
@@ -767,24 +827,33 @@
         <v>0.2696472943125345</v>
       </c>
       <c r="H7" t="n">
+        <v>0.3129324682495859</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.5133114301490889</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.3494873274434014</v>
+      </c>
+      <c r="K7" t="n">
         <v>0.2411282856401674</v>
       </c>
-      <c r="I7" t="n">
+      <c r="L7" t="n">
         <v>10.49855072463768</v>
       </c>
-      <c r="J7" t="n">
+      <c r="M7" t="n">
         <v>8.255072463768116</v>
       </c>
-      <c r="K7" t="n">
+      <c r="N7" t="n">
         <v>9.376811594202898</v>
       </c>
-      <c r="L7" t="n">
+      <c r="O7" t="n">
         <v>3.23768115942029</v>
       </c>
-      <c r="M7" t="n">
+      <c r="P7" t="n">
         <v>1.843478260869565</v>
       </c>
-      <c r="N7" t="n">
+      <c r="Q7" t="n">
         <v>0.6461144927536232</v>
       </c>
     </row>
@@ -817,24 +886,33 @@
         <v>0.3363377685696746</v>
       </c>
       <c r="H8" t="n">
+        <v>0.3641314149785144</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.523633855125844</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.4211070748925722</v>
+      </c>
+      <c r="K8" t="n">
         <v>0.1782244636783564</v>
       </c>
-      <c r="I8" t="n">
+      <c r="L8" t="n">
         <v>18.88695652173913</v>
       </c>
-      <c r="J8" t="n">
+      <c r="M8" t="n">
         <v>13.2231884057971</v>
       </c>
-      <c r="K8" t="n">
+      <c r="N8" t="n">
         <v>15.2231884057971</v>
       </c>
-      <c r="L8" t="n">
+      <c r="O8" t="n">
         <v>7.371014492753623</v>
       </c>
-      <c r="M8" t="n">
+      <c r="P8" t="n">
         <v>4.388405797101449</v>
       </c>
-      <c r="N8" t="n">
+      <c r="Q8" t="n">
         <v>0.6492246376811595</v>
       </c>
     </row>
@@ -867,24 +945,33 @@
         <v>0.3123173669467787</v>
       </c>
       <c r="H9" t="n">
+        <v>0.2850038935574229</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.4282945098039216</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.3934320168067227</v>
+      </c>
+      <c r="K9" t="n">
         <v>0.2793174385013324</v>
       </c>
-      <c r="I9" t="n">
+      <c r="L9" t="n">
         <v>10.37790697674419</v>
       </c>
-      <c r="J9" t="n">
+      <c r="M9" t="n">
         <v>8.572674418604651</v>
       </c>
-      <c r="K9" t="n">
+      <c r="N9" t="n">
         <v>9.212209302325581</v>
       </c>
-      <c r="L9" t="n">
+      <c r="O9" t="n">
         <v>2.962209302325582</v>
       </c>
-      <c r="M9" t="n">
+      <c r="P9" t="n">
         <v>1.86046511627907</v>
       </c>
-      <c r="N9" t="n">
+      <c r="Q9" t="n">
         <v>0.5934212209302325</v>
       </c>
     </row>
@@ -917,24 +1004,33 @@
         <v>0.4283139776665383</v>
       </c>
       <c r="H10" t="n">
+        <v>0.416978629187524</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.555167577974586</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.6152305737389295</v>
+      </c>
+      <c r="K10" t="n">
         <v>0.3869941211670341</v>
       </c>
-      <c r="I10" t="n">
+      <c r="L10" t="n">
         <v>15.05507246376812</v>
       </c>
-      <c r="J10" t="n">
+      <c r="M10" t="n">
         <v>11.46086956521739</v>
       </c>
-      <c r="K10" t="n">
+      <c r="N10" t="n">
         <v>11.87826086956522</v>
       </c>
-      <c r="L10" t="n">
+      <c r="O10" t="n">
         <v>4.524637681159421</v>
       </c>
-      <c r="M10" t="n">
+      <c r="P10" t="n">
         <v>3.852173913043478</v>
       </c>
-      <c r="N10" t="n">
+      <c r="Q10" t="n">
         <v>0.7440411594202898</v>
       </c>
     </row>
@@ -967,24 +1063,33 @@
         <v>0.4172204790419162</v>
       </c>
       <c r="H11" t="n">
+        <v>0.409197125748503</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.6059871457085828</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.5325052694610778</v>
+      </c>
+      <c r="K11" t="n">
         <v>0.502428598994489</v>
       </c>
-      <c r="I11" t="n">
+      <c r="L11" t="n">
         <v>7.303206997084548</v>
       </c>
-      <c r="J11" t="n">
+      <c r="M11" t="n">
         <v>6.142857142857143</v>
       </c>
-      <c r="K11" t="n">
+      <c r="N11" t="n">
         <v>6.699708454810495</v>
       </c>
-      <c r="L11" t="n">
+      <c r="O11" t="n">
         <v>1.982507288629738</v>
       </c>
-      <c r="M11" t="n">
+      <c r="P11" t="n">
         <v>1.297376093294461</v>
       </c>
-      <c r="N11" t="n">
+      <c r="Q11" t="n">
         <v>0.6472160349854227</v>
       </c>
     </row>
@@ -1017,24 +1122,33 @@
         <v>0.3925871423647018</v>
       </c>
       <c r="H12" t="n">
+        <v>0.4231451913133402</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.6802644605308514</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.508275008617718</v>
+      </c>
+      <c r="K12" t="n">
         <v>0.4464035657963256</v>
       </c>
-      <c r="I12" t="n">
+      <c r="L12" t="n">
         <v>8.408695652173913</v>
       </c>
-      <c r="J12" t="n">
+      <c r="M12" t="n">
         <v>7.298550724637681</v>
       </c>
-      <c r="K12" t="n">
+      <c r="N12" t="n">
         <v>7.397101449275362</v>
       </c>
-      <c r="L12" t="n">
+      <c r="O12" t="n">
         <v>1.942028985507246</v>
       </c>
-      <c r="M12" t="n">
+      <c r="P12" t="n">
         <v>1.681159420289855</v>
       </c>
-      <c r="N12" t="n">
+      <c r="Q12" t="n">
         <v>0.6742495652173913</v>
       </c>
     </row>
@@ -1067,24 +1181,33 @@
         <v>0.3286145465429512</v>
       </c>
       <c r="H13" t="n">
+        <v>0.3815840167614487</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.5939462436396289</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.4509010176593834</v>
+      </c>
+      <c r="K13" t="n">
         <v>0.2106986864979593</v>
       </c>
-      <c r="I13" t="n">
+      <c r="L13" t="n">
         <v>19.36811594202899</v>
       </c>
-      <c r="J13" t="n">
+      <c r="M13" t="n">
         <v>14.6</v>
       </c>
-      <c r="K13" t="n">
+      <c r="N13" t="n">
         <v>16.19130434782609</v>
       </c>
-      <c r="L13" t="n">
+      <c r="O13" t="n">
         <v>5.669565217391304</v>
       </c>
-      <c r="M13" t="n">
+      <c r="P13" t="n">
         <v>3.933333333333333</v>
       </c>
-      <c r="N13" t="n">
+      <c r="Q13" t="n">
         <v>0.6207594202898551</v>
       </c>
     </row>
@@ -1117,24 +1240,33 @@
         <v>0.278065910808768</v>
       </c>
       <c r="H14" t="n">
+        <v>0.279756462585034</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.4885729906777526</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.3895644998740237</v>
+      </c>
+      <c r="K14" t="n">
         <v>0.2978285013678073</v>
       </c>
-      <c r="I14" t="n">
+      <c r="L14" t="n">
         <v>11.50434782608696</v>
       </c>
-      <c r="J14" t="n">
+      <c r="M14" t="n">
         <v>9.466666666666667</v>
       </c>
-      <c r="K14" t="n">
+      <c r="N14" t="n">
         <v>10.39710144927536</v>
       </c>
-      <c r="L14" t="n">
+      <c r="O14" t="n">
         <v>2.802898550724638</v>
       </c>
-      <c r="M14" t="n">
+      <c r="P14" t="n">
         <v>1.878260869565217</v>
       </c>
-      <c r="N14" t="n">
+      <c r="Q14" t="n">
         <v>0.5621771014492754</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated scores: accepted icd10 codes -> jaccard and diagnostic checklist
</commit_message>
<xml_diff>
--- a/saved/run_batch_20260912/analysis/v4_metrics_summary_plain.xlsx
+++ b/saved/run_batch_20260912/analysis/v4_metrics_summary_plain.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="28">
   <si>
     <t>patient</t>
   </si>
@@ -64,7 +64,10 @@
     <t>overcommitment_conf</t>
   </si>
   <si>
-    <t>diagnostic_reasoning_overall_score</t>
+    <t>diagnostic_evidence_sufficiency_gt</t>
+  </si>
+  <si>
+    <t>diagnostic_evidence_sufficiency_pred</t>
   </si>
   <si>
     <t>gemini-3.1-pro-preview</t>
@@ -144,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -153,9 +156,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -466,29 +466,30 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -540,37 +541,40 @@
       <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D2" s="3">
-        <v>62.89855072463768</v>
+        <v>69.56521739130434</v>
       </c>
       <c r="E2" s="3">
-        <v>0.3024618969298246</v>
+        <v>0.3212944353070176</v>
       </c>
       <c r="F2" s="3">
-        <v>0.5621556743421052</v>
+        <v>0.5870507127192982</v>
       </c>
       <c r="G2" s="3">
-        <v>0.415893475877193</v>
+        <v>0.4516730537280702</v>
       </c>
       <c r="H2" s="3">
-        <v>0.3792011513157895</v>
+        <v>0.3969475603070176</v>
       </c>
       <c r="I2" s="3">
-        <v>0.5264231359649123</v>
+        <v>0.5480058114035088</v>
       </c>
       <c r="J2" s="3">
-        <v>0.534404221491228</v>
+        <v>0.574977576754386</v>
       </c>
       <c r="K2" s="3">
         <v>0.4161504717057321</v>
@@ -582,30 +586,33 @@
         <v>8.15072463768116</v>
       </c>
       <c r="N2" s="3">
-        <v>8.86376811594203</v>
+        <v>8.495652173913044</v>
       </c>
       <c r="O2" s="3">
         <v>3.568115942028986</v>
       </c>
       <c r="P2" s="3">
-        <v>2.365217391304348</v>
+        <v>2.701449275362319</v>
       </c>
       <c r="Q2" s="3">
         <v>0.7026315942028986</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
+      <c r="R2" s="3">
+        <v>0.7371057228915663</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
       <c r="A3" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D3" s="3">
-        <v>59.1304347826087</v>
+        <v>62.89855072463768</v>
       </c>
       <c r="E3" s="3">
         <v>0.3295659776902887</v>
@@ -643,40 +650,39 @@
       <c r="P3" s="3">
         <v>2.150724637681159</v>
       </c>
-      <c r="Q3" s="3">
-        <v>0.691099420289855</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D4" s="3">
-        <v>66.08695652173913</v>
+        <v>73.6231884057971</v>
       </c>
       <c r="E4" s="3">
-        <v>0.3233745905474965</v>
+        <v>0.3553535329901731</v>
       </c>
       <c r="F4" s="3">
-        <v>0.6444472157229761</v>
+        <v>0.7060685540477305</v>
       </c>
       <c r="G4" s="3">
-        <v>0.3917180627047263</v>
+        <v>0.4302771174543753</v>
       </c>
       <c r="H4" s="3">
-        <v>0.3967591951333646</v>
+        <v>0.423094244267665</v>
       </c>
       <c r="I4" s="3">
-        <v>0.5684520355638746</v>
+        <v>0.6111991109031353</v>
       </c>
       <c r="J4" s="3">
-        <v>0.512912915301825</v>
+        <v>0.5514313523631259</v>
       </c>
       <c r="K4" s="3">
         <v>0.463501933647481</v>
@@ -688,30 +694,33 @@
         <v>5.704347826086956</v>
       </c>
       <c r="N4" s="3">
-        <v>5.87536231884058</v>
+        <v>5.666666666666667</v>
       </c>
       <c r="O4" s="3">
         <v>1.385507246376812</v>
       </c>
       <c r="P4" s="3">
-        <v>0.9739130434782609</v>
+        <v>1.147826086956522</v>
       </c>
       <c r="Q4" s="3">
         <v>0.6727484057971015</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
+      <c r="R4" s="3">
+        <v>0.7203921686746988</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
       <c r="A5" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D5" s="3">
-        <v>66.08695652173913</v>
+        <v>70.14492753623189</v>
       </c>
       <c r="E5" s="3">
         <v>0.3267175311620426</v>
@@ -749,40 +758,39 @@
       <c r="P5" s="3">
         <v>1.478260869565217</v>
       </c>
-      <c r="Q5" s="3">
-        <v>0.6466733333333333</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
       <c r="A6" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D6" s="3">
-        <v>71.8840579710145</v>
+        <v>75.3623188405797</v>
       </c>
       <c r="E6" s="3">
-        <v>0.3745598744769875</v>
+        <v>0.3845720920502092</v>
       </c>
       <c r="F6" s="3">
-        <v>0.7039676150627615</v>
+        <v>0.7134098326359832</v>
       </c>
       <c r="G6" s="3">
-        <v>0.4316124686192468</v>
+        <v>0.4480679916317992</v>
       </c>
       <c r="H6" s="3">
-        <v>0.4298293723849372</v>
+        <v>0.4360441422594142</v>
       </c>
       <c r="I6" s="3">
-        <v>0.6505427615062761</v>
+        <v>0.6562820083682008</v>
       </c>
       <c r="J6" s="3">
-        <v>0.5154064435146444</v>
+        <v>0.530587489539749</v>
       </c>
       <c r="K6" s="3">
         <v>0.4584506540095213</v>
@@ -794,30 +802,33 @@
         <v>5.855072463768116</v>
       </c>
       <c r="N6" s="3">
-        <v>5.991304347826087</v>
+        <v>5.921739130434783</v>
       </c>
       <c r="O6" s="3">
         <v>1.776811594202899</v>
       </c>
       <c r="P6" s="3">
-        <v>1.542028985507246</v>
+        <v>1.6</v>
       </c>
       <c r="Q6" s="3">
         <v>0.6801655072463768</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
+      <c r="R6" s="3">
+        <v>0.7155879518072289</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="4">
-        <v>40</v>
+        <v>24</v>
+      </c>
+      <c r="D7" s="3">
+        <v>51.59420289855073</v>
       </c>
       <c r="E7" s="3">
         <v>0.2484040309221425</v>
@@ -855,40 +866,39 @@
       <c r="P7" s="3">
         <v>1.843478260869565</v>
       </c>
-      <c r="Q7" s="3">
-        <v>0.6461144927536232</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D8" s="3">
-        <v>40.8695652173913</v>
+        <v>45.79710144927536</v>
       </c>
       <c r="E8" s="3">
-        <v>0.2930542817679558</v>
+        <v>0.3200106046654389</v>
       </c>
       <c r="F8" s="3">
-        <v>0.5599546807857582</v>
+        <v>0.5833586402701043</v>
       </c>
       <c r="G8" s="3">
-        <v>0.3363377685696746</v>
+        <v>0.3741493554327808</v>
       </c>
       <c r="H8" s="3">
-        <v>0.3641314149785144</v>
+        <v>0.3928008287292818</v>
       </c>
       <c r="I8" s="3">
-        <v>0.523633855125844</v>
+        <v>0.5452857427869858</v>
       </c>
       <c r="J8" s="3">
-        <v>0.4211070748925722</v>
+        <v>0.4631662369551872</v>
       </c>
       <c r="K8" s="3">
         <v>0.1782244636783564</v>
@@ -900,48 +910,51 @@
         <v>13.2231884057971</v>
       </c>
       <c r="N8" s="3">
-        <v>15.2231884057971</v>
+        <v>14.60289855072464</v>
       </c>
       <c r="O8" s="3">
         <v>7.371014492753623</v>
       </c>
       <c r="P8" s="3">
-        <v>4.388405797101449</v>
+        <v>4.976811594202899</v>
       </c>
       <c r="Q8" s="3">
         <v>0.6492246376811595</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
+      <c r="R8" s="3">
+        <v>0.6482441558441558</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
       <c r="A9" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D9" s="3">
-        <v>46.22093023255814</v>
+        <v>50.58139534883721</v>
       </c>
       <c r="E9" s="3">
-        <v>0.2411692717086835</v>
+        <v>0.2648810364145658</v>
       </c>
       <c r="F9" s="3">
-        <v>0.4900498319327731</v>
+        <v>0.5119456302521008</v>
       </c>
       <c r="G9" s="3">
-        <v>0.3123173669467787</v>
+        <v>0.3484120168067227</v>
       </c>
       <c r="H9" s="3">
-        <v>0.2850038935574229</v>
+        <v>0.3097026050420168</v>
       </c>
       <c r="I9" s="3">
-        <v>0.4282945098039216</v>
+        <v>0.4457555182072829</v>
       </c>
       <c r="J9" s="3">
-        <v>0.3934320168067227</v>
+        <v>0.4373490756302521</v>
       </c>
       <c r="K9" s="3">
         <v>0.2793174385013324</v>
@@ -953,48 +966,51 @@
         <v>8.57267441860465</v>
       </c>
       <c r="N9" s="3">
-        <v>9.212209302325581</v>
+        <v>8.991279069767442</v>
       </c>
       <c r="O9" s="3">
         <v>2.962209302325582</v>
       </c>
       <c r="P9" s="3">
-        <v>1.86046511627907</v>
+        <v>2.052325581395349</v>
       </c>
       <c r="Q9" s="3">
         <v>0.5934212209302325</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18">
+      <c r="R9" s="3">
+        <v>0.5874517799352751</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
       <c r="A10" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D10" s="3">
-        <v>68.69565217391305</v>
+        <v>73.91304347826087</v>
       </c>
       <c r="E10" s="3">
-        <v>0.3158201771274547</v>
+        <v>0.3253985367731999</v>
       </c>
       <c r="F10" s="3">
-        <v>0.6538400462071621</v>
+        <v>0.6653474971120523</v>
       </c>
       <c r="G10" s="3">
-        <v>0.4283139776665383</v>
+        <v>0.4579071236041586</v>
       </c>
       <c r="H10" s="3">
-        <v>0.416978629187524</v>
+        <v>0.4192948016942626</v>
       </c>
       <c r="I10" s="3">
-        <v>0.555167577974586</v>
+        <v>0.5624821909896034</v>
       </c>
       <c r="J10" s="3">
-        <v>0.6152305737389295</v>
+        <v>0.6425984405082787</v>
       </c>
       <c r="K10" s="3">
         <v>0.3869941211670341</v>
@@ -1006,48 +1022,51 @@
         <v>11.46086956521739</v>
       </c>
       <c r="N10" s="3">
-        <v>11.87826086956522</v>
+        <v>11.58260869565217</v>
       </c>
       <c r="O10" s="3">
         <v>4.524637681159421</v>
       </c>
       <c r="P10" s="3">
-        <v>3.852173913043478</v>
+        <v>4.127536231884058</v>
       </c>
       <c r="Q10" s="3">
         <v>0.7440411594202898</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18">
+      <c r="R10" s="3">
+        <v>0.7839948328267478</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
       <c r="A11" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D11" s="3">
-        <v>61.80758017492711</v>
+        <v>71.13702623906705</v>
       </c>
       <c r="E11" s="3">
-        <v>0.3343255089820359</v>
+        <v>0.3650610379241517</v>
       </c>
       <c r="F11" s="3">
-        <v>0.6538584031936128</v>
+        <v>0.7281239920159681</v>
       </c>
       <c r="G11" s="3">
-        <v>0.4172204790419162</v>
+        <v>0.4543394411177645</v>
       </c>
       <c r="H11" s="3">
-        <v>0.409197125748503</v>
+        <v>0.4372708982035928</v>
       </c>
       <c r="I11" s="3">
-        <v>0.6059871457085828</v>
+        <v>0.6581164471057884</v>
       </c>
       <c r="J11" s="3">
-        <v>0.5325052694610778</v>
+        <v>0.5708455489021956</v>
       </c>
       <c r="K11" s="3">
         <v>0.502428598994489</v>
@@ -1059,48 +1078,51 @@
         <v>6.142857142857143</v>
       </c>
       <c r="N11" s="3">
-        <v>6.699708454810495</v>
+        <v>6.12536443148688</v>
       </c>
       <c r="O11" s="3">
         <v>1.982507288629738</v>
       </c>
       <c r="P11" s="3">
-        <v>1.297376093294461</v>
+        <v>1.833819241982507</v>
       </c>
       <c r="Q11" s="3">
         <v>0.6472160349854227</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18">
+      <c r="R11" s="3">
+        <v>0.692938905775076</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
       <c r="A12" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D12" s="3">
-        <v>71.30434782608695</v>
+        <v>74.78260869565217</v>
       </c>
       <c r="E12" s="3">
-        <v>0.3443259565667011</v>
+        <v>0.3552864874181317</v>
       </c>
       <c r="F12" s="3">
-        <v>0.7618919682867976</v>
+        <v>0.781919510513616</v>
       </c>
       <c r="G12" s="3">
-        <v>0.3925871423647018</v>
+        <v>0.4071324370906584</v>
       </c>
       <c r="H12" s="3">
-        <v>0.4231451913133402</v>
+        <v>0.4333336091003102</v>
       </c>
       <c r="I12" s="3">
-        <v>0.6802644605308514</v>
+        <v>0.698045742847294</v>
       </c>
       <c r="J12" s="3">
-        <v>0.508275008617718</v>
+        <v>0.5242939331265081</v>
       </c>
       <c r="K12" s="3">
         <v>0.4464035657963256</v>
@@ -1112,7 +1134,7 @@
         <v>7.298550724637681</v>
       </c>
       <c r="N12" s="3">
-        <v>7.397101449275362</v>
+        <v>7.394202898550724</v>
       </c>
       <c r="O12" s="3">
         <v>1.942028985507246</v>
@@ -1123,37 +1145,40 @@
       <c r="Q12" s="3">
         <v>0.6742495652173913</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18">
+      <c r="R12" s="3">
+        <v>0.6970002994011976</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
       <c r="A13" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D13" s="3">
-        <v>38.84057971014493</v>
+        <v>41.44927536231884</v>
       </c>
       <c r="E13" s="3">
-        <v>0.29232014366956</v>
+        <v>0.3157756210715355</v>
       </c>
       <c r="F13" s="3">
-        <v>0.681707123615684</v>
+        <v>0.6903621370847052</v>
       </c>
       <c r="G13" s="3">
-        <v>0.3286145465429512</v>
+        <v>0.3575665219994014</v>
       </c>
       <c r="H13" s="3">
-        <v>0.3815840167614487</v>
+        <v>0.3994010924872792</v>
       </c>
       <c r="I13" s="3">
-        <v>0.5939462436396289</v>
+        <v>0.6026010475905418</v>
       </c>
       <c r="J13" s="3">
-        <v>0.4509010176593834</v>
+        <v>0.4786712810535768</v>
       </c>
       <c r="K13" s="3">
         <v>0.2106986864979593</v>
@@ -1165,48 +1190,51 @@
         <v>14.6</v>
       </c>
       <c r="N13" s="3">
-        <v>16.19130434782609</v>
+        <v>15.8463768115942</v>
       </c>
       <c r="O13" s="3">
         <v>5.669565217391304</v>
       </c>
       <c r="P13" s="3">
-        <v>3.933333333333333</v>
+        <v>4.260869565217392</v>
       </c>
       <c r="Q13" s="3">
         <v>0.6207594202898551</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18">
+      <c r="R13" s="3">
+        <v>0.6219019867549669</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
       <c r="A14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="D14" s="3">
-        <v>40.8695652173913</v>
+        <v>46.08695652173913</v>
       </c>
       <c r="E14" s="3">
-        <v>0.2236265054169816</v>
+        <v>0.2403937011841774</v>
       </c>
       <c r="F14" s="3">
-        <v>0.5587509952129</v>
+        <v>0.5733952884857647</v>
       </c>
       <c r="G14" s="3">
-        <v>0.278065910808768</v>
+        <v>0.3081016124968506</v>
       </c>
       <c r="H14" s="3">
-        <v>0.279756462585034</v>
+        <v>0.2932850088183421</v>
       </c>
       <c r="I14" s="3">
-        <v>0.4885729906777526</v>
+        <v>0.4977110355253213</v>
       </c>
       <c r="J14" s="3">
-        <v>0.3895644998740237</v>
+        <v>0.4200843285462333</v>
       </c>
       <c r="K14" s="3">
         <v>0.2978285013678073</v>
@@ -1218,16 +1246,19 @@
         <v>9.466666666666667</v>
       </c>
       <c r="N14" s="3">
-        <v>10.39710144927536</v>
+        <v>10.14202898550725</v>
       </c>
       <c r="O14" s="3">
         <v>2.802898550724638</v>
       </c>
       <c r="P14" s="3">
-        <v>1.878260869565217</v>
+        <v>2.092753623188406</v>
       </c>
       <c r="Q14" s="3">
         <v>0.5621771014492754</v>
+      </c>
+      <c r="R14" s="3">
+        <v>0.5440190625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>